<commit_message>
Auto Update Daily Reports: 2026/06/26 週五  8:46:35.29
</commit_message>
<xml_diff>
--- a/資產_20260601.xlsx
+++ b/資產_20260601.xlsx
@@ -5,14 +5,15 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2026\alex\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2025\AI\MongoDB\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12270"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12270" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="工作表1" sheetId="1" r:id="rId1"/>
+    <sheet name="差異分析" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="164">
   <si>
     <t>股票</t>
   </si>
@@ -343,6 +344,215 @@
   </si>
   <si>
     <t>台東成功土地</t>
+  </si>
+  <si>
+    <t>資產差異分析：2026/1/17 vs 2026/7/1</t>
+  </si>
+  <si>
+    <t>項目</t>
+  </si>
+  <si>
+    <t>差異</t>
+  </si>
+  <si>
+    <t>說明</t>
+  </si>
+  <si>
+    <t>總資產（表列計）</t>
+  </si>
+  <si>
+    <t>差距 $3,703,955</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>原因說明</t>
+  </si>
+  <si>
+    <t>富邦房貸（新增負債）</t>
+  </si>
+  <si>
+    <t>施羅德六年期（2025到期）</t>
+  </si>
+  <si>
+    <t>CRO（加密貨幣）</t>
+  </si>
+  <si>
+    <t>加密貨幣市值下跌</t>
+  </si>
+  <si>
+    <t>小幅減少</t>
+  </si>
+  <si>
+    <t>▲ 拉高總計的項目</t>
+  </si>
+  <si>
+    <t>永豐日本基金（原大戶日本基金）</t>
+  </si>
+  <si>
+    <t>公司互助會（新增）</t>
+  </si>
+  <si>
+    <t>7/1 新增項目</t>
+  </si>
+  <si>
+    <t>Schwab美股（新增）</t>
+  </si>
+  <si>
+    <t>永豐美股（新增）</t>
+  </si>
+  <si>
+    <t>小幅增加</t>
+  </si>
+  <si>
+    <t>1/17 項目</t>
+  </si>
+  <si>
+    <t>7/1 對應項目</t>
+  </si>
+  <si>
+    <t>股票+豐存股+統一證券</t>
+  </si>
+  <si>
+    <t>凱基證+統一證+大戶投</t>
+  </si>
+  <si>
+    <t>股票部位整體增加 +$257,608</t>
+  </si>
+  <si>
+    <t>共同投資(美股)</t>
+  </si>
+  <si>
+    <t>不明（Schwab? 永豐美股?）</t>
+  </si>
+  <si>
+    <t>合併後餘額反而增加</t>
+  </si>
+  <si>
+    <t>超商禮券</t>
+  </si>
+  <si>
+    <t>名稱更新，金額相同</t>
+  </si>
+  <si>
+    <t>差異彙整</t>
+  </si>
+  <si>
+    <t>可辨識減少小計</t>
+  </si>
+  <si>
+    <t>可辨識增加小計</t>
+  </si>
+  <si>
+    <t>■ 總覽</t>
+  </si>
+  <si>
+    <t>不動產（7/1新增，未估值）</t>
+  </si>
+  <si>
+    <t>汐止觀止 ＋ 台東成功土地</t>
+  </si>
+  <si>
+    <t>若計入市值，7/1 實際總資產應高於 $13,102,521</t>
+  </si>
+  <si>
+    <t>▼ 拖低總計的主要原因（確定項目）</t>
+  </si>
+  <si>
+    <t>1/17 無此項；7/1 計入房貸負債，直接扣減總資產</t>
+  </si>
+  <si>
+    <t>大戶外幣（美+日幣）</t>
+  </si>
+  <si>
+    <t>日幣$27,105+美金$985,769 → 合計縮水近半，匯率損失或資金移出</t>
+  </si>
+  <si>
+    <t>2025已到期應已領回，7/1 空白，資金去向待確認</t>
+  </si>
+  <si>
+    <t>7/1 改為國泰投資型保險基金，金額大幅縮水</t>
+  </si>
+  <si>
+    <t>小幅下降</t>
+  </si>
+  <si>
+    <t>小計（確定減少）</t>
+  </si>
+  <si>
+    <t>資金大量集中到中信，大幅增加</t>
+  </si>
+  <si>
+    <t>從大戶轉至永豐，金額增加 +$302,786</t>
+  </si>
+  <si>
+    <t>新增美股帳戶（可能來自共同投資美股$500k轉換）</t>
+  </si>
+  <si>
+    <t>新增美股部位，大幅擴充美股投資</t>
+  </si>
+  <si>
+    <t>市值小幅增加</t>
+  </si>
+  <si>
+    <t>小計（確定增加）</t>
+  </si>
+  <si>
+    <r>
+      <t>◈</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="新細明體"/>
+        <family val="1"/>
+        <charset val="136"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 帳戶結構重組（難以直接對應）</t>
+    </r>
+  </si>
+  <si>
+    <t>1/17 金額</t>
+  </si>
+  <si>
+    <t>7/1 金額</t>
+  </si>
+  <si>
+    <t>消失，可能清算或轉帳戶，建議確認</t>
+  </si>
+  <si>
+    <t>大戶外幣(日幣+美金)</t>
+  </si>
+  <si>
+    <t>合併後大幅縮水 -$461,510</t>
+  </si>
+  <si>
+    <t>⚠  注意事項 / 建議追蹤</t>
+  </si>
+  <si>
+    <t>① 汐止觀止 及 台東成功土地：7/1 新增不動產項目，尚未填入估值。若計入市值，總資產實際高於 $13,102,521。</t>
+  </si>
+  <si>
+    <t>② 施羅德六年期 $204,600（2025到期）：7/1 欄位空白，應已領回。建議確認入帳位置。</t>
+  </si>
+  <si>
+    <t>③ 共同投資(美股) $500,000：7/1 消失，建議確認是否清算、轉入 Schwab 或永豐美股。</t>
+  </si>
+  <si>
+    <t>④ 大戶外幣缺口 -$461,510：建議確認是匯率損失（日圓/美元貶值）或已移轉至他處。</t>
+  </si>
+  <si>
+    <t>⑤ 加密貨幣（CRO + 幣安）：共下跌 $213,797，反映市值波動，非資金移出。</t>
+  </si>
+  <si>
+    <t>總計實際差異</t>
+  </si>
+  <si>
+    <t>其餘差距（結構重組/未追蹤）</t>
   </si>
 </sst>
 </file>
@@ -352,9 +562,9 @@
   <numFmts count="3">
     <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0;[Red]\-&quot;$&quot;#,##0"/>
     <numFmt numFmtId="176" formatCode="&quot;$&quot;#,##0"/>
-    <numFmt numFmtId="182" formatCode="&quot;NT$&quot;#,##0_);\(&quot;NT$&quot;#,##0\)"/>
+    <numFmt numFmtId="177" formatCode="&quot;NT$&quot;#,##0_);\(&quot;NT$&quot;#,##0\)"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="12">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -420,8 +630,35 @@
       <charset val="136"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="新細明體"/>
+      <family val="1"/>
+      <charset val="136"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="新細明體"/>
+      <family val="2"/>
+      <charset val="136"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="1"/>
+      <name val="新細明體"/>
+      <family val="1"/>
+      <charset val="136"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="19">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -452,8 +689,86 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0000C0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE0E0FF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCCCCFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF235637"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDAEFE2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCEEFC6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7F3C5B"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFE6F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF008FBF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC0FFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF854124"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE4DCD6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF64381F"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="8">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -564,6 +879,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
@@ -573,7 +903,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -610,7 +940,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -636,6 +966,87 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="8" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="8" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="8" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="17" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="17" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="8" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="8" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="8" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="11" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -965,7 +1376,7 @@
         <v>155383</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="32" thickBot="1">
+    <row r="4" spans="1:5" ht="17.5" thickBot="1">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -979,7 +1390,7 @@
         <v>1399733</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="32" thickBot="1">
+    <row r="5" spans="1:5" ht="17.5" thickBot="1">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -993,7 +1404,7 @@
         <v>700000</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="32" thickBot="1">
+    <row r="6" spans="1:5" ht="17.5" thickBot="1">
       <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
@@ -1007,7 +1418,7 @@
         <v>978284</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="47.5" thickBot="1">
+    <row r="7" spans="1:5" ht="17.5" thickBot="1">
       <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
@@ -1045,7 +1456,7 @@
       <c r="D9" s="13"/>
       <c r="E9" s="14"/>
     </row>
-    <row r="10" spans="1:5" ht="51.5" thickBot="1">
+    <row r="10" spans="1:5" ht="17.5" thickBot="1">
       <c r="A10" s="3" t="s">
         <v>7</v>
       </c>
@@ -1059,7 +1470,7 @@
         <v>49673</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="34.5" thickBot="1">
+    <row r="11" spans="1:5" ht="17.5" thickBot="1">
       <c r="A11" s="3" t="s">
         <v>8</v>
       </c>
@@ -1073,7 +1484,7 @@
         <v>33821</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="34.5" thickBot="1">
+    <row r="12" spans="1:5" ht="17.5" thickBot="1">
       <c r="A12" s="5" t="s">
         <v>9</v>
       </c>
@@ -1087,7 +1498,7 @@
         <v>25289</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="34.5" thickBot="1">
+    <row r="13" spans="1:5" ht="17.5" thickBot="1">
       <c r="A13" s="5" t="s">
         <v>10</v>
       </c>
@@ -1101,7 +1512,7 @@
         <v>-670151</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="34.5" thickBot="1">
+    <row r="14" spans="1:5" ht="17.5" thickBot="1">
       <c r="A14" s="5" t="s">
         <v>11</v>
       </c>
@@ -1115,7 +1526,7 @@
         <v>2088663</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="34.5" thickBot="1">
+    <row r="15" spans="1:5" ht="17.5" thickBot="1">
       <c r="A15" s="5" t="s">
         <v>12</v>
       </c>
@@ -1129,7 +1540,7 @@
         <v>5168</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="34.5" thickBot="1">
+    <row r="16" spans="1:5" ht="17.5" thickBot="1">
       <c r="A16" s="5" t="s">
         <v>13</v>
       </c>
@@ -1143,7 +1554,7 @@
         <v>74347</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="34.5" thickBot="1">
+    <row r="17" spans="1:5" ht="17.5" thickBot="1">
       <c r="A17" s="5" t="s">
         <v>14</v>
       </c>
@@ -1157,7 +1568,7 @@
         <v>7829</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="34.5" thickBot="1">
+    <row r="18" spans="1:5" ht="17.5" thickBot="1">
       <c r="A18" s="5" t="s">
         <v>15</v>
       </c>
@@ -1171,7 +1582,7 @@
         <v>1025</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="34.5" thickBot="1">
+    <row r="19" spans="1:5" ht="17.5" thickBot="1">
       <c r="A19" s="5" t="s">
         <v>16</v>
       </c>
@@ -1183,7 +1594,7 @@
       </c>
       <c r="E19" s="14"/>
     </row>
-    <row r="20" spans="1:5" ht="34.5" thickBot="1">
+    <row r="20" spans="1:5" ht="17.5" thickBot="1">
       <c r="A20" s="5" t="s">
         <v>17</v>
       </c>
@@ -1197,7 +1608,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="34.5" thickBot="1">
+    <row r="21" spans="1:5" ht="17.5" thickBot="1">
       <c r="A21" s="5" t="s">
         <v>18</v>
       </c>
@@ -1211,7 +1622,7 @@
         <v>23955</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="34.5" thickBot="1">
+    <row r="22" spans="1:5" ht="17.5" thickBot="1">
       <c r="A22" s="3" t="s">
         <v>19</v>
       </c>
@@ -1225,7 +1636,7 @@
         <v>39465</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="34.5" thickBot="1">
+    <row r="23" spans="1:5" ht="17.5" thickBot="1">
       <c r="A23" s="3" t="s">
         <v>20</v>
       </c>
@@ -1239,7 +1650,7 @@
         <v>116535</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="51.5" thickBot="1">
+    <row r="24" spans="1:5" ht="17.5" thickBot="1">
       <c r="A24" s="3" t="s">
         <v>21</v>
       </c>
@@ -1253,7 +1664,7 @@
         <v>551364</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="34.5" thickBot="1">
+    <row r="25" spans="1:5" ht="17.5" thickBot="1">
       <c r="A25" s="3" t="s">
         <v>22</v>
       </c>
@@ -1267,7 +1678,7 @@
         <v>595521</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="34.5" thickBot="1">
+    <row r="26" spans="1:5" ht="17.5" thickBot="1">
       <c r="A26" s="3" t="s">
         <v>23</v>
       </c>
@@ -1281,7 +1692,7 @@
         <v>83126</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="51.5" thickBot="1">
+    <row r="27" spans="1:5" ht="17.5" thickBot="1">
       <c r="A27" s="3" t="s">
         <v>24</v>
       </c>
@@ -1295,7 +1706,7 @@
         <v>336416</v>
       </c>
     </row>
-    <row r="28" spans="1:5" ht="34.5" thickBot="1">
+    <row r="28" spans="1:5" ht="17.5" thickBot="1">
       <c r="A28" s="3" t="s">
         <v>25</v>
       </c>
@@ -1309,7 +1720,7 @@
         <v>758</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="34.5" thickBot="1">
+    <row r="29" spans="1:5" ht="17.5" thickBot="1">
       <c r="A29" s="3" t="s">
         <v>26</v>
       </c>
@@ -1333,7 +1744,7 @@
       <c r="D30" s="13"/>
       <c r="E30" s="14"/>
     </row>
-    <row r="31" spans="1:5" ht="68.5" thickBot="1">
+    <row r="31" spans="1:5" ht="34.5" thickBot="1">
       <c r="A31" s="6" t="s">
         <v>28</v>
       </c>
@@ -1347,7 +1758,7 @@
         <v>644436</v>
       </c>
     </row>
-    <row r="32" spans="1:5" ht="68.5" thickBot="1">
+    <row r="32" spans="1:5" ht="17.5" thickBot="1">
       <c r="A32" s="6" t="s">
         <v>29</v>
       </c>
@@ -1361,7 +1772,7 @@
         <v>217868</v>
       </c>
     </row>
-    <row r="33" spans="1:5" ht="68.5" thickBot="1">
+    <row r="33" spans="1:5" ht="17.5" thickBot="1">
       <c r="A33" s="6" t="s">
         <v>30</v>
       </c>
@@ -1375,7 +1786,7 @@
         <v>245550</v>
       </c>
     </row>
-    <row r="34" spans="1:5" ht="68.5" thickBot="1">
+    <row r="34" spans="1:5" ht="17.5" thickBot="1">
       <c r="A34" s="6" t="s">
         <v>31</v>
       </c>
@@ -1389,7 +1800,7 @@
         <v>171620</v>
       </c>
     </row>
-    <row r="35" spans="1:5" ht="51.5" thickBot="1">
+    <row r="35" spans="1:5" ht="17.5" thickBot="1">
       <c r="A35" s="6" t="s">
         <v>32</v>
       </c>
@@ -1403,7 +1814,7 @@
         <v>337497</v>
       </c>
     </row>
-    <row r="36" spans="1:5" ht="68.5" thickBot="1">
+    <row r="36" spans="1:5" ht="34.5" thickBot="1">
       <c r="A36" s="6" t="s">
         <v>33</v>
       </c>
@@ -1415,7 +1826,7 @@
       </c>
       <c r="E36" s="14"/>
     </row>
-    <row r="37" spans="1:5" ht="102.5" thickBot="1">
+    <row r="37" spans="1:5" ht="34.5" thickBot="1">
       <c r="A37" s="6" t="s">
         <v>34</v>
       </c>
@@ -1429,7 +1840,7 @@
         <v>351564</v>
       </c>
     </row>
-    <row r="38" spans="1:5" ht="51.5" thickBot="1">
+    <row r="38" spans="1:5" ht="34.5" thickBot="1">
       <c r="A38" s="6" t="s">
         <v>35</v>
       </c>
@@ -1443,7 +1854,7 @@
         <v>882516</v>
       </c>
     </row>
-    <row r="39" spans="1:5" ht="51.5" thickBot="1">
+    <row r="39" spans="1:5" ht="17.5" thickBot="1">
       <c r="A39" s="6" t="s">
         <v>36</v>
       </c>
@@ -1457,7 +1868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:5" ht="68.5" thickBot="1">
+    <row r="40" spans="1:5" ht="17.5" thickBot="1">
       <c r="A40" s="6" t="s">
         <v>37</v>
       </c>
@@ -1471,7 +1882,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:5" ht="85.5" thickBot="1">
+    <row r="41" spans="1:5" ht="34.5" thickBot="1">
       <c r="A41" s="6" t="s">
         <v>38</v>
       </c>
@@ -1485,7 +1896,7 @@
         <v>724999</v>
       </c>
     </row>
-    <row r="42" spans="1:5" ht="68.5" thickBot="1">
+    <row r="42" spans="1:5" ht="17.5" thickBot="1">
       <c r="A42" s="6" t="s">
         <v>39</v>
       </c>
@@ -1499,7 +1910,7 @@
         <v>1314540</v>
       </c>
     </row>
-    <row r="43" spans="1:5" ht="85.5" thickBot="1">
+    <row r="43" spans="1:5" ht="34.5" thickBot="1">
       <c r="A43" s="6" t="s">
         <v>40</v>
       </c>
@@ -1513,7 +1924,7 @@
         <v>1028385</v>
       </c>
     </row>
-    <row r="44" spans="1:5" ht="51.5" thickBot="1">
+    <row r="44" spans="1:5" ht="17.5" thickBot="1">
       <c r="A44" s="6" t="s">
         <v>41</v>
       </c>
@@ -1547,7 +1958,7 @@
       <c r="D46" s="13"/>
       <c r="E46" s="14"/>
     </row>
-    <row r="47" spans="1:5" ht="51.5" thickBot="1">
+    <row r="47" spans="1:5" ht="17.5" thickBot="1">
       <c r="A47" s="6" t="s">
         <v>44</v>
       </c>
@@ -1561,7 +1972,7 @@
         <v>4069</v>
       </c>
     </row>
-    <row r="48" spans="1:5" ht="34.5" thickBot="1">
+    <row r="48" spans="1:5" ht="17.5" thickBot="1">
       <c r="A48" s="6" t="s">
         <v>45</v>
       </c>
@@ -1659,7 +2070,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:5" ht="34.5" thickBot="1">
+    <row r="55" spans="1:5" ht="17.5" thickBot="1">
       <c r="A55" s="6" t="s">
         <v>52</v>
       </c>
@@ -1687,7 +2098,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="57" spans="1:5" ht="32" thickBot="1">
+    <row r="57" spans="1:5" ht="17.5" thickBot="1">
       <c r="A57" s="6" t="s">
         <v>54</v>
       </c>
@@ -1725,7 +2136,7 @@
         <v>240000</v>
       </c>
     </row>
-    <row r="60" spans="1:5" ht="34.5" thickBot="1">
+    <row r="60" spans="1:5" ht="17.5" thickBot="1">
       <c r="A60" s="6" t="s">
         <v>57</v>
       </c>
@@ -1739,7 +2150,7 @@
         <v>13000</v>
       </c>
     </row>
-    <row r="61" spans="1:5" ht="34.5" thickBot="1">
+    <row r="61" spans="1:5" ht="17.5" thickBot="1">
       <c r="A61" s="6" t="s">
         <v>58</v>
       </c>
@@ -1781,7 +2192,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="64" spans="1:5" ht="34.5" thickBot="1">
+    <row r="64" spans="1:5" ht="17.5" thickBot="1">
       <c r="A64" s="6" t="s">
         <v>61</v>
       </c>
@@ -1860,7 +2271,7 @@
         <v>230000</v>
       </c>
     </row>
-    <row r="72" spans="1:5" ht="34.5" thickBot="1">
+    <row r="72" spans="1:5" ht="17.5" thickBot="1">
       <c r="D72" s="15" t="s">
         <v>95</v>
       </c>
@@ -1868,7 +2279,7 @@
         <v>1076668</v>
       </c>
     </row>
-    <row r="73" spans="1:5" ht="47.5" thickBot="1">
+    <row r="73" spans="1:5" ht="17.5" thickBot="1">
       <c r="D73" s="11" t="s">
         <v>96</v>
       </c>
@@ -1876,13 +2287,13 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="74" spans="1:5" ht="31.5" thickBot="1">
+    <row r="74" spans="1:5" ht="17.5" thickBot="1">
       <c r="D74" s="11" t="s">
         <v>97</v>
       </c>
       <c r="E74" s="14"/>
     </row>
-    <row r="75" spans="1:5" ht="31.5" thickBot="1">
+    <row r="75" spans="1:5" ht="17.5" thickBot="1">
       <c r="D75" s="11" t="s">
         <v>98</v>
       </c>
@@ -1906,4 +2317,639 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E50"/>
+  <sheetFormatPr defaultRowHeight="17"/>
+  <cols>
+    <col min="1" max="1" width="36.6328125" customWidth="1"/>
+    <col min="2" max="2" width="15.6328125" customWidth="1"/>
+    <col min="3" max="3" width="32.6328125" customWidth="1"/>
+    <col min="4" max="4" width="15.6328125" customWidth="1"/>
+    <col min="5" max="5" width="55.6328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="34" customHeight="1">
+      <c r="A1" s="32" t="s">
+        <v>99</v>
+      </c>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+    </row>
+    <row r="3" spans="1:5" ht="22" customHeight="1">
+      <c r="A3" s="33" t="s">
+        <v>132</v>
+      </c>
+      <c r="B3" s="31"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="34" t="s">
+        <v>100</v>
+      </c>
+      <c r="B4" s="35">
+        <v>46039</v>
+      </c>
+      <c r="C4" s="35">
+        <v>46204</v>
+      </c>
+      <c r="D4" s="34" t="s">
+        <v>101</v>
+      </c>
+      <c r="E4" s="34" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="21" t="s">
+        <v>103</v>
+      </c>
+      <c r="B5" s="36">
+        <v>16806476</v>
+      </c>
+      <c r="C5" s="36">
+        <v>13102521</v>
+      </c>
+      <c r="D5" s="29">
+        <v>-3703955</v>
+      </c>
+      <c r="E5" s="21" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="B6" s="23" t="s">
+        <v>105</v>
+      </c>
+      <c r="C6" s="21" t="s">
+        <v>134</v>
+      </c>
+      <c r="D6" s="23" t="s">
+        <v>105</v>
+      </c>
+      <c r="E6" s="21" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="22" customHeight="1">
+      <c r="A8" s="37" t="s">
+        <v>136</v>
+      </c>
+      <c r="B8" s="31"/>
+      <c r="C8" s="31"/>
+      <c r="D8" s="31"/>
+      <c r="E8" s="31"/>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="34" t="s">
+        <v>100</v>
+      </c>
+      <c r="B9" s="35">
+        <v>46039</v>
+      </c>
+      <c r="C9" s="35">
+        <v>46204</v>
+      </c>
+      <c r="D9" s="34" t="s">
+        <v>101</v>
+      </c>
+      <c r="E9" s="34" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="24" t="s">
+        <v>107</v>
+      </c>
+      <c r="B10" s="22">
+        <v>0</v>
+      </c>
+      <c r="C10" s="22">
+        <v>-670151</v>
+      </c>
+      <c r="D10" s="29">
+        <v>-670151</v>
+      </c>
+      <c r="E10" s="21" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" s="24" t="s">
+        <v>138</v>
+      </c>
+      <c r="B11" s="22">
+        <v>1012874</v>
+      </c>
+      <c r="C11" s="22">
+        <v>551364</v>
+      </c>
+      <c r="D11" s="29">
+        <v>-461510</v>
+      </c>
+      <c r="E11" s="21" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="24" t="s">
+        <v>108</v>
+      </c>
+      <c r="B12" s="22">
+        <v>204600</v>
+      </c>
+      <c r="C12" s="22">
+        <v>0</v>
+      </c>
+      <c r="D12" s="29">
+        <v>-204600</v>
+      </c>
+      <c r="E12" s="21" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="24" t="s">
+        <v>109</v>
+      </c>
+      <c r="B13" s="22">
+        <v>503285</v>
+      </c>
+      <c r="C13" s="22">
+        <v>320910</v>
+      </c>
+      <c r="D13" s="29">
+        <v>-182375</v>
+      </c>
+      <c r="E13" s="21" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" s="24" t="s">
+        <v>1</v>
+      </c>
+      <c r="B14" s="22">
+        <v>217214</v>
+      </c>
+      <c r="C14" s="22">
+        <v>67589</v>
+      </c>
+      <c r="D14" s="29">
+        <v>-149625</v>
+      </c>
+      <c r="E14" s="21" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" s="24" t="s">
+        <v>95</v>
+      </c>
+      <c r="B15" s="22">
+        <v>1140859</v>
+      </c>
+      <c r="C15" s="22">
+        <v>1076668</v>
+      </c>
+      <c r="D15" s="29">
+        <v>-64191</v>
+      </c>
+      <c r="E15" s="21" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" s="24" t="s">
+        <v>91</v>
+      </c>
+      <c r="B16" s="22">
+        <v>93031</v>
+      </c>
+      <c r="C16" s="22">
+        <v>61609</v>
+      </c>
+      <c r="D16" s="29">
+        <v>-31422</v>
+      </c>
+      <c r="E16" s="21" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" s="22">
+        <v>2118861</v>
+      </c>
+      <c r="C17" s="22">
+        <v>2088663</v>
+      </c>
+      <c r="D17" s="29">
+        <v>-30198</v>
+      </c>
+      <c r="E17" s="21" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" s="25" t="s">
+        <v>143</v>
+      </c>
+      <c r="B18" s="38"/>
+      <c r="C18" s="38"/>
+      <c r="D18" s="39">
+        <v>-1794072</v>
+      </c>
+      <c r="E18" s="38"/>
+    </row>
+    <row r="20" spans="1:5" ht="22" customHeight="1">
+      <c r="A20" s="40" t="s">
+        <v>112</v>
+      </c>
+      <c r="B20" s="31"/>
+      <c r="C20" s="31"/>
+      <c r="D20" s="31"/>
+      <c r="E20" s="31"/>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" s="34" t="s">
+        <v>100</v>
+      </c>
+      <c r="B21" s="35">
+        <v>46039</v>
+      </c>
+      <c r="C21" s="35">
+        <v>46204</v>
+      </c>
+      <c r="D21" s="34" t="s">
+        <v>101</v>
+      </c>
+      <c r="E21" s="34" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22" s="26" t="s">
+        <v>6</v>
+      </c>
+      <c r="B22" s="22">
+        <v>97643</v>
+      </c>
+      <c r="C22" s="22">
+        <v>595521</v>
+      </c>
+      <c r="D22" s="29">
+        <v>497878</v>
+      </c>
+      <c r="E22" s="21" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23" s="26" t="s">
+        <v>113</v>
+      </c>
+      <c r="B23" s="22">
+        <v>675498</v>
+      </c>
+      <c r="C23" s="22">
+        <v>978284</v>
+      </c>
+      <c r="D23" s="29">
+        <v>302786</v>
+      </c>
+      <c r="E23" s="21" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5">
+      <c r="A24" s="26" t="s">
+        <v>114</v>
+      </c>
+      <c r="B24" s="22">
+        <v>0</v>
+      </c>
+      <c r="C24" s="22">
+        <v>300000</v>
+      </c>
+      <c r="D24" s="29">
+        <v>300000</v>
+      </c>
+      <c r="E24" s="21" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25" s="26" t="s">
+        <v>116</v>
+      </c>
+      <c r="B25" s="22">
+        <v>0</v>
+      </c>
+      <c r="C25" s="22">
+        <v>700000</v>
+      </c>
+      <c r="D25" s="29">
+        <v>700000</v>
+      </c>
+      <c r="E25" s="21" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26" s="26" t="s">
+        <v>117</v>
+      </c>
+      <c r="B26" s="22">
+        <v>0</v>
+      </c>
+      <c r="C26" s="22">
+        <v>1399733</v>
+      </c>
+      <c r="D26" s="29">
+        <v>1399733</v>
+      </c>
+      <c r="E26" s="21" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="A27" s="26" t="s">
+        <v>94</v>
+      </c>
+      <c r="B27" s="22">
+        <v>200000</v>
+      </c>
+      <c r="C27" s="22">
+        <v>230000</v>
+      </c>
+      <c r="D27" s="29">
+        <v>30000</v>
+      </c>
+      <c r="E27" s="21" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28" s="26" t="s">
+        <v>52</v>
+      </c>
+      <c r="B28" s="22">
+        <v>311767</v>
+      </c>
+      <c r="C28" s="22">
+        <v>319956</v>
+      </c>
+      <c r="D28" s="29">
+        <v>8189</v>
+      </c>
+      <c r="E28" s="21" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29" s="27" t="s">
+        <v>149</v>
+      </c>
+      <c r="B29" s="41"/>
+      <c r="C29" s="41"/>
+      <c r="D29" s="42">
+        <v>3238586</v>
+      </c>
+      <c r="E29" s="41"/>
+    </row>
+    <row r="31" spans="1:5" ht="22" customHeight="1">
+      <c r="A31" s="43" t="s">
+        <v>150</v>
+      </c>
+      <c r="B31" s="31"/>
+      <c r="C31" s="31"/>
+      <c r="D31" s="31"/>
+      <c r="E31" s="31"/>
+    </row>
+    <row r="32" spans="1:5">
+      <c r="A32" s="34" t="s">
+        <v>119</v>
+      </c>
+      <c r="B32" s="34" t="s">
+        <v>151</v>
+      </c>
+      <c r="C32" s="34" t="s">
+        <v>120</v>
+      </c>
+      <c r="D32" s="34" t="s">
+        <v>152</v>
+      </c>
+      <c r="E32" s="34" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5">
+      <c r="A33" s="28" t="s">
+        <v>121</v>
+      </c>
+      <c r="B33" s="22">
+        <v>2936711</v>
+      </c>
+      <c r="C33" s="21" t="s">
+        <v>122</v>
+      </c>
+      <c r="D33" s="22">
+        <v>3194319</v>
+      </c>
+      <c r="E33" s="21" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5">
+      <c r="A34" s="28" t="s">
+        <v>124</v>
+      </c>
+      <c r="B34" s="22">
+        <v>500000</v>
+      </c>
+      <c r="C34" s="21" t="s">
+        <v>125</v>
+      </c>
+      <c r="D34" s="44" t="s">
+        <v>105</v>
+      </c>
+      <c r="E34" s="21" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5">
+      <c r="A35" s="28" t="s">
+        <v>154</v>
+      </c>
+      <c r="B35" s="22">
+        <v>1012874</v>
+      </c>
+      <c r="C35" s="21" t="s">
+        <v>77</v>
+      </c>
+      <c r="D35" s="22">
+        <v>551364</v>
+      </c>
+      <c r="E35" s="21" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5">
+      <c r="A36" s="28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B36" s="22">
+        <v>14331</v>
+      </c>
+      <c r="C36" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="D36" s="22">
+        <v>62727</v>
+      </c>
+      <c r="E36" s="21" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5">
+      <c r="A37" s="28" t="s">
+        <v>127</v>
+      </c>
+      <c r="B37" s="22">
+        <v>240000</v>
+      </c>
+      <c r="C37" s="21" t="s">
+        <v>85</v>
+      </c>
+      <c r="D37" s="22">
+        <v>240000</v>
+      </c>
+      <c r="E37" s="21" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="22" customHeight="1">
+      <c r="A40" s="45" t="s">
+        <v>156</v>
+      </c>
+      <c r="B40" s="31"/>
+      <c r="C40" s="31"/>
+      <c r="D40" s="31"/>
+      <c r="E40" s="31"/>
+    </row>
+    <row r="41" spans="1:5" ht="30" customHeight="1">
+      <c r="A41" s="30" t="s">
+        <v>157</v>
+      </c>
+      <c r="B41" s="46"/>
+      <c r="C41" s="46"/>
+      <c r="D41" s="46"/>
+      <c r="E41" s="46"/>
+    </row>
+    <row r="42" spans="1:5" ht="30" customHeight="1">
+      <c r="A42" s="30" t="s">
+        <v>158</v>
+      </c>
+      <c r="B42" s="46"/>
+      <c r="C42" s="46"/>
+      <c r="D42" s="46"/>
+      <c r="E42" s="46"/>
+    </row>
+    <row r="43" spans="1:5" ht="30" customHeight="1">
+      <c r="A43" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="B43" s="46"/>
+      <c r="C43" s="46"/>
+      <c r="D43" s="46"/>
+      <c r="E43" s="46"/>
+    </row>
+    <row r="44" spans="1:5" ht="30" customHeight="1">
+      <c r="A44" s="30" t="s">
+        <v>160</v>
+      </c>
+      <c r="B44" s="46"/>
+      <c r="C44" s="46"/>
+      <c r="D44" s="46"/>
+      <c r="E44" s="46"/>
+    </row>
+    <row r="45" spans="1:5" ht="30" customHeight="1">
+      <c r="A45" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="B45" s="46"/>
+      <c r="C45" s="46"/>
+      <c r="D45" s="46"/>
+      <c r="E45" s="46"/>
+    </row>
+    <row r="48" spans="1:5" ht="22" customHeight="1">
+      <c r="A48" s="47" t="s">
+        <v>129</v>
+      </c>
+      <c r="B48" s="31"/>
+      <c r="C48" s="31"/>
+      <c r="D48" s="31"/>
+      <c r="E48" s="31"/>
+    </row>
+    <row r="49" spans="1:5">
+      <c r="A49" s="21" t="s">
+        <v>130</v>
+      </c>
+      <c r="B49" s="29">
+        <v>-1794072</v>
+      </c>
+      <c r="C49" s="21" t="s">
+        <v>131</v>
+      </c>
+      <c r="D49" s="29">
+        <v>3238586</v>
+      </c>
+      <c r="E49" s="21"/>
+    </row>
+    <row r="50" spans="1:5">
+      <c r="A50" s="21" t="s">
+        <v>162</v>
+      </c>
+      <c r="B50" s="29">
+        <v>-3703955</v>
+      </c>
+      <c r="C50" s="21" t="s">
+        <v>163</v>
+      </c>
+      <c r="D50" s="29">
+        <v>5148469</v>
+      </c>
+      <c r="E50" s="21"/>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="A41:E41"/>
+    <mergeCell ref="A42:E42"/>
+    <mergeCell ref="A43:E43"/>
+    <mergeCell ref="A44:E44"/>
+    <mergeCell ref="A45:E45"/>
+    <mergeCell ref="A48:E48"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A8:E8"/>
+    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A31:E31"/>
+    <mergeCell ref="A40:E40"/>
+  </mergeCells>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>